<commit_message>
Add WFD thresholds to plots
</commit_message>
<xml_diff>
--- a/data/vann-nett_data.xlsx
+++ b/data/vann-nett_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P79"/>
+  <dimension ref="A1:P65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -943,7 +943,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>002-3899-R</t>
+          <t>002-3891-R</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -963,17 +963,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Bad</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.1024</v>
+        <v>0.0133</v>
       </c>
       <c r="G9" t="n">
-        <v>0.4072</v>
+        <v>0.0426</v>
       </c>
       <c r="H9" t="n">
-        <v>97.67</v>
+        <v>750</v>
       </c>
       <c r="I9" t="n">
         <v>10</v>
@@ -989,13 +989,13 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="M9" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="N9" t="n">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1011,7 +1011,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>002-3899-R</t>
+          <t>002-3891-R</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1035,13 +1035,13 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.3825</v>
+        <v>0.2492</v>
       </c>
       <c r="G10" t="n">
-        <v>0.5576</v>
+        <v>0.4045</v>
       </c>
       <c r="H10" t="n">
-        <v>849.763285</v>
+        <v>1304.204932</v>
       </c>
       <c r="I10" t="n">
         <v>325</v>
@@ -1057,13 +1057,13 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="M10" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="N10" t="n">
-        <v>207</v>
+        <v>148</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1079,7 +1079,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>002-3899-R</t>
+          <t>002-3891-R</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1105,7 +1105,7 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>7.331736</v>
+        <v>6.89</v>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
@@ -1115,13 +1115,13 @@
       </c>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="M11" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="N11" t="n">
-        <v>167</v>
+        <v>74</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1137,7 +1137,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>002-3899-R</t>
+          <t>002-3891-R</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1147,23 +1147,25 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>QE3-1-6-1 - Nitrogen conditions</t>
+          <t>QE3-1-6-2 - Phosphorus Conditions</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Total oxidised Nitrogen</t>
+          <t>Orthophosphate</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Not classified</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
+      <c r="G12" t="n">
+        <v>0.5</v>
+      </c>
       <c r="H12" t="n">
-        <v>543.166666</v>
+        <v>24</v>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
@@ -1173,13 +1175,13 @@
       </c>
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="M12" t="n">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="N12" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1195,7 +1197,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>002-3899-R</t>
+          <t>002-3891-R</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1210,7 +1212,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Orthophosphate</t>
+          <t>Total phosphorous</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1223,23 +1225,23 @@
         <v>0.5</v>
       </c>
       <c r="H13" t="n">
-        <v>42.089655</v>
+        <v>45.919601</v>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
-          <t>µg/l</t>
+          <t>µg/l P</t>
         </is>
       </c>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="M13" t="n">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="N13" t="n">
-        <v>29</v>
+        <v>148</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1255,7 +1257,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>002-3899-R</t>
+          <t>002-3891-R</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1270,36 +1272,34 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Total phosphorous</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Not classified</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
-      <c r="G14" t="n">
-        <v>0.5</v>
-      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
-        <v>42.583091</v>
+        <v>13.330612</v>
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
-          <t>µg/l P</t>
+          <t>µg/l</t>
         </is>
       </c>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="M14" t="n">
         <v>2025</v>
       </c>
       <c r="N14" t="n">
-        <v>207</v>
+        <v>49</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1315,7 +1315,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>002-3899-R</t>
+          <t>002-1638-R</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1325,39 +1325,49 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>QE3-1-6-2 - Phosphorus Conditions</t>
+          <t>QE3-1-6-1 - Nitrogen conditions</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Phosphate</t>
+          <t>Ammonia</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Not classified</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
+          <t>Bad</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.0864</v>
+      </c>
       <c r="H15" t="n">
-        <v>21.361206</v>
-      </c>
-      <c r="I15" t="inlineStr"/>
+        <v>371</v>
+      </c>
+      <c r="I15" t="n">
+        <v>10</v>
+      </c>
       <c r="J15" t="inlineStr">
         <is>
           <t>µg/l</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>30.0;60.0;100.0;160.0</t>
+        </is>
+      </c>
       <c r="L15" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="M15" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="N15" t="n">
-        <v>116</v>
+        <v>22</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1373,7 +1383,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>002-3891-R</t>
+          <t>002-1638-R</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1388,25 +1398,25 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Ammonia</t>
+          <t>Total nitrogen</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Bad</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.0133</v>
+        <v>0.3546</v>
       </c>
       <c r="G16" t="n">
-        <v>0.0426</v>
+        <v>0.5256</v>
       </c>
       <c r="H16" t="n">
-        <v>750</v>
+        <v>916.619805</v>
       </c>
       <c r="I16" t="n">
-        <v>10</v>
+        <v>325</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -1415,7 +1425,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>30.0;60.0;100.0;160.0</t>
+          <t>550.0;775.0;1325.0;2025.0</t>
         </is>
       </c>
       <c r="L16" t="n">
@@ -1425,7 +1435,7 @@
         <v>2026</v>
       </c>
       <c r="N16" t="n">
-        <v>46</v>
+        <v>103</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1441,7 +1451,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>002-3891-R</t>
+          <t>002-1638-R</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1456,36 +1466,26 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Total nitrogen</t>
+          <t>Total organic carbon</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="F17" t="n">
-        <v>0.2492</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0.4045</v>
-      </c>
+          <t>Not classified</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
-        <v>1304.204932</v>
-      </c>
-      <c r="I17" t="n">
-        <v>325</v>
-      </c>
+        <v>6.029864</v>
+      </c>
+      <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
-          <t>µg/l</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>550.0;775.0;1325.0;2025.0</t>
-        </is>
-      </c>
+          <t>mg/l C</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="n">
         <v>2020</v>
       </c>
@@ -1493,7 +1493,7 @@
         <v>2026</v>
       </c>
       <c r="N17" t="n">
-        <v>148</v>
+        <v>74</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1509,7 +1509,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>002-3891-R</t>
+          <t>002-1638-R</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Total organic carbon</t>
+          <t>Total oxidised Nitrogen</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1535,23 +1535,23 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>6.89</v>
+        <v>413.75</v>
       </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
-          <t>mg/l C</t>
+          <t>µg/l</t>
         </is>
       </c>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="n">
-        <v>2020</v>
+        <v>2025</v>
       </c>
       <c r="M18" t="n">
         <v>2026</v>
       </c>
       <c r="N18" t="n">
-        <v>74</v>
+        <v>8</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1567,7 +1567,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>002-3891-R</t>
+          <t>002-1638-R</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1595,7 +1595,7 @@
         <v>0.5</v>
       </c>
       <c r="H19" t="n">
-        <v>24</v>
+        <v>14.305263</v>
       </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr">
@@ -1608,10 +1608,10 @@
         <v>2020</v>
       </c>
       <c r="M19" t="n">
-        <v>2020</v>
+        <v>2026</v>
       </c>
       <c r="N19" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1627,7 +1627,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>002-3891-R</t>
+          <t>002-1638-R</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1647,15 +1647,15 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="H20" t="n">
-        <v>45.919601</v>
+        <v>32.305631</v>
       </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr">
@@ -1671,7 +1671,7 @@
         <v>2026</v>
       </c>
       <c r="N20" t="n">
-        <v>148</v>
+        <v>103</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -1687,7 +1687,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>002-3891-R</t>
+          <t>002-1638-R</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1713,7 +1713,7 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>13.330612</v>
+        <v>10.06</v>
       </c>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
@@ -1723,13 +1723,13 @@
       </c>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="M21" t="n">
         <v>2025</v>
       </c>
       <c r="N21" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -1745,7 +1745,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>002-1638-R</t>
+          <t>002-3384-R</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1769,13 +1769,13 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0.027</v>
+        <v>0.0294</v>
       </c>
       <c r="G22" t="n">
-        <v>0.0864</v>
+        <v>0.0941</v>
       </c>
       <c r="H22" t="n">
-        <v>371</v>
+        <v>340</v>
       </c>
       <c r="I22" t="n">
         <v>10</v>
@@ -1794,10 +1794,10 @@
         <v>2020</v>
       </c>
       <c r="M22" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="N22" t="n">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
@@ -1813,7 +1813,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>002-1638-R</t>
+          <t>002-3384-R</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1837,13 +1837,13 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>0.3546</v>
+        <v>0.2874</v>
       </c>
       <c r="G23" t="n">
-        <v>0.5256</v>
+        <v>0.4484</v>
       </c>
       <c r="H23" t="n">
-        <v>916.619805</v>
+        <v>1131.018018</v>
       </c>
       <c r="I23" t="n">
         <v>325</v>
@@ -1859,13 +1859,13 @@
         </is>
       </c>
       <c r="L23" t="n">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="M23" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="N23" t="n">
-        <v>103</v>
+        <v>222</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -1881,7 +1881,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>002-1638-R</t>
+          <t>002-3384-R</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1907,7 +1907,7 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>6.029864</v>
+        <v>7.045181</v>
       </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr">
@@ -1917,13 +1917,13 @@
       </c>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="n">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="M24" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="N24" t="n">
-        <v>74</v>
+        <v>220</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -1939,7 +1939,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>002-1638-R</t>
+          <t>002-3384-R</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1965,7 +1965,7 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
-        <v>413.75</v>
+        <v>593.423076</v>
       </c>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
@@ -1975,13 +1975,13 @@
       </c>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="n">
-        <v>2025</v>
+        <v>2020</v>
       </c>
       <c r="M25" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="N25" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -1997,7 +1997,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>002-1638-R</t>
+          <t>002-3384-R</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2025,7 +2025,7 @@
         <v>0.5</v>
       </c>
       <c r="H26" t="n">
-        <v>14.305263</v>
+        <v>49.459433</v>
       </c>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
@@ -2035,13 +2035,13 @@
       </c>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="n">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="M26" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="N26" t="n">
-        <v>19</v>
+        <v>106</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2057,7 +2057,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>002-1638-R</t>
+          <t>002-3384-R</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2077,15 +2077,15 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="H27" t="n">
-        <v>32.305631</v>
+        <v>74.41351299999999</v>
       </c>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
@@ -2095,13 +2095,13 @@
       </c>
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="n">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="M27" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="N27" t="n">
-        <v>103</v>
+        <v>222</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2117,7 +2117,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>002-1638-R</t>
+          <t>002-3384-R</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2143,7 +2143,7 @@
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>10.06</v>
+        <v>67.552941</v>
       </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr">
@@ -2153,13 +2153,13 @@
       </c>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="M28" t="n">
         <v>2025</v>
       </c>
       <c r="N28" t="n">
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -2175,7 +2175,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>002-3384-R</t>
+          <t>002-3659-R</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2195,17 +2195,17 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Bad</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>0.0294</v>
+        <v>0.0893</v>
       </c>
       <c r="G29" t="n">
-        <v>0.0941</v>
+        <v>0.3429</v>
       </c>
       <c r="H29" t="n">
-        <v>340</v>
+        <v>112</v>
       </c>
       <c r="I29" t="n">
         <v>10</v>
@@ -2221,17 +2221,15 @@
         </is>
       </c>
       <c r="L29" t="n">
-        <v>2020</v>
+        <v>2014</v>
       </c>
       <c r="M29" t="n">
-        <v>2025</v>
-      </c>
-      <c r="N29" t="n">
-        <v>31</v>
-      </c>
+        <v>2014</v>
+      </c>
+      <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Vannmiljø</t>
+          <t>WATERENVIRONMENT_SFTDN</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -2243,7 +2241,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>002-3384-R</t>
+          <t>002-3659-R</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2263,17 +2261,17 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>0.2874</v>
+        <v>0.1624</v>
       </c>
       <c r="G30" t="n">
-        <v>0.4484</v>
+        <v>0.2045</v>
       </c>
       <c r="H30" t="n">
-        <v>1131.018018</v>
+        <v>2001.248648</v>
       </c>
       <c r="I30" t="n">
         <v>325</v>
@@ -2289,13 +2287,13 @@
         </is>
       </c>
       <c r="L30" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="M30" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="N30" t="n">
-        <v>222</v>
+        <v>185</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -2311,7 +2309,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>002-3384-R</t>
+          <t>002-3659-R</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2337,7 +2335,7 @@
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>7.045181</v>
+        <v>11.558152</v>
       </c>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
@@ -2347,13 +2345,13 @@
       </c>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="M31" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="N31" t="n">
-        <v>220</v>
+        <v>184</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -2369,7 +2367,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>002-3384-R</t>
+          <t>002-3659-R</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2395,7 +2393,7 @@
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>593.423076</v>
+        <v>1227.5</v>
       </c>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr">
@@ -2405,17 +2403,15 @@
       </c>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="n">
-        <v>2020</v>
+        <v>2014</v>
       </c>
       <c r="M32" t="n">
-        <v>2023</v>
-      </c>
-      <c r="N32" t="n">
-        <v>26</v>
-      </c>
+        <v>2014</v>
+      </c>
+      <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Vannmiljø</t>
+          <t>WATERENVIRONMENT_SFTDN</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
@@ -2427,7 +2423,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>002-3384-R</t>
+          <t>002-3659-R</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2447,15 +2443,13 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Not classified</t>
         </is>
       </c>
       <c r="F33" t="inlineStr"/>
-      <c r="G33" t="n">
-        <v>0.5</v>
-      </c>
+      <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
-        <v>49.459433</v>
+        <v>46.070588</v>
       </c>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
@@ -2465,13 +2459,13 @@
       </c>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="M33" t="n">
         <v>2025</v>
       </c>
       <c r="N33" t="n">
-        <v>106</v>
+        <v>68</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
@@ -2487,7 +2481,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>002-3384-R</t>
+          <t>002-3659-R</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2507,15 +2501,15 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="H34" t="n">
-        <v>74.41351299999999</v>
+        <v>94.451612</v>
       </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr">
@@ -2525,13 +2519,13 @@
       </c>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="M34" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="N34" t="n">
-        <v>222</v>
+        <v>186</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
@@ -2547,7 +2541,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>002-3384-R</t>
+          <t>002-3659-R</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2573,7 +2567,7 @@
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
-        <v>67.552941</v>
+        <v>67.820212</v>
       </c>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
@@ -2583,13 +2577,13 @@
       </c>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="n">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="M35" t="n">
         <v>2025</v>
       </c>
       <c r="N35" t="n">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
@@ -2605,7 +2599,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>002-3384-R</t>
+          <t>002-599-R</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2625,17 +2619,17 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Bad</t>
+          <t>Poor</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>0.0294</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="G36" t="n">
-        <v>0.0941</v>
+        <v>0.2347</v>
       </c>
       <c r="H36" t="n">
-        <v>340</v>
+        <v>145</v>
       </c>
       <c r="I36" t="n">
         <v>10</v>
@@ -2651,13 +2645,13 @@
         </is>
       </c>
       <c r="L36" t="n">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="M36" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="N36" t="n">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
@@ -2673,7 +2667,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>002-3384-R</t>
+          <t>002-599-R</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2693,17 +2687,17 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Bad</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>0.2874</v>
+        <v>0.1229</v>
       </c>
       <c r="G37" t="n">
-        <v>0.4484</v>
+        <v>0.1531</v>
       </c>
       <c r="H37" t="n">
-        <v>1131.018018</v>
+        <v>2645.257731</v>
       </c>
       <c r="I37" t="n">
         <v>325</v>
@@ -2725,7 +2719,7 @@
         <v>2025</v>
       </c>
       <c r="N37" t="n">
-        <v>222</v>
+        <v>97</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
@@ -2741,7 +2735,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>002-3384-R</t>
+          <t>002-599-R</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2767,7 +2761,7 @@
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
-        <v>7.045181</v>
+        <v>9.52</v>
       </c>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr">
@@ -2783,7 +2777,7 @@
         <v>2025</v>
       </c>
       <c r="N38" t="n">
-        <v>220</v>
+        <v>91</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
@@ -2799,7 +2793,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>002-3384-R</t>
+          <t>002-599-R</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2825,7 +2819,7 @@
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="n">
-        <v>593.423076</v>
+        <v>1578.333333</v>
       </c>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
@@ -2835,13 +2829,13 @@
       </c>
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="n">
-        <v>2020</v>
+        <v>2022</v>
       </c>
       <c r="M39" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="N39" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
@@ -2857,7 +2851,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>002-3384-R</t>
+          <t>002-599-R</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2885,7 +2879,7 @@
         <v>0.5</v>
       </c>
       <c r="H40" t="n">
-        <v>49.459433</v>
+        <v>60.289473</v>
       </c>
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr">
@@ -2898,10 +2892,10 @@
         <v>2019</v>
       </c>
       <c r="M40" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="N40" t="n">
-        <v>106</v>
+        <v>38</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
@@ -2917,7 +2911,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>002-3384-R</t>
+          <t>002-599-R</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2945,7 +2939,7 @@
         <v>0.5</v>
       </c>
       <c r="H41" t="n">
-        <v>74.41351299999999</v>
+        <v>83.15000000000001</v>
       </c>
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr">
@@ -2961,7 +2955,7 @@
         <v>2025</v>
       </c>
       <c r="N41" t="n">
-        <v>222</v>
+        <v>100</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
@@ -2977,7 +2971,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>002-3384-R</t>
+          <t>002-599-R</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3003,7 +2997,7 @@
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="n">
-        <v>67.552941</v>
+        <v>65.61764700000001</v>
       </c>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr">
@@ -3019,7 +3013,7 @@
         <v>2025</v>
       </c>
       <c r="N42" t="n">
-        <v>85</v>
+        <v>34</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
@@ -3035,7 +3029,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>002-3659-R</t>
+          <t>002-3685-R</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3055,17 +3049,17 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>0.0893</v>
+        <v>0.1524</v>
       </c>
       <c r="G43" t="n">
-        <v>0.3429</v>
+        <v>0.5571</v>
       </c>
       <c r="H43" t="n">
-        <v>112</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="I43" t="n">
         <v>10</v>
@@ -3089,7 +3083,7 @@
       <c r="N43" t="inlineStr"/>
       <c r="O43" t="inlineStr">
         <is>
-          <t>WATERENVIRONMENT_SFTDN</t>
+          <t>VannMiljø</t>
         </is>
       </c>
       <c r="P43" t="inlineStr">
@@ -3101,7 +3095,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>002-3659-R</t>
+          <t>002-3685-R</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3121,17 +3115,17 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>0.1624</v>
+        <v>0.2474</v>
       </c>
       <c r="G44" t="n">
-        <v>0.2045</v>
+        <v>0.4024</v>
       </c>
       <c r="H44" t="n">
-        <v>2001.248648</v>
+        <v>1313.451612</v>
       </c>
       <c r="I44" t="n">
         <v>325</v>
@@ -3153,7 +3147,7 @@
         <v>2026</v>
       </c>
       <c r="N44" t="n">
-        <v>185</v>
+        <v>124</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
@@ -3169,7 +3163,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>002-3659-R</t>
+          <t>002-3685-R</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3184,7 +3178,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Total organic carbon</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -3195,12 +3189,12 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="n">
-        <v>11.558152</v>
+        <v>34.871028</v>
       </c>
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
-          <t>mg/l C</t>
+          <t>µg/l</t>
         </is>
       </c>
       <c r="K45" t="inlineStr"/>
@@ -3208,10 +3202,10 @@
         <v>2020</v>
       </c>
       <c r="M45" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="N45" t="n">
-        <v>184</v>
+        <v>107</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
@@ -3227,7 +3221,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>002-3659-R</t>
+          <t>002-3685-R</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3242,7 +3236,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Total oxidised Nitrogen</t>
+          <t>Total organic carbon</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -3253,25 +3247,27 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="n">
-        <v>1227.5</v>
+        <v>13.990163</v>
       </c>
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr">
         <is>
-          <t>µg/l</t>
+          <t>mg/l C</t>
         </is>
       </c>
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="n">
-        <v>2014</v>
+        <v>2020</v>
       </c>
       <c r="M46" t="n">
-        <v>2014</v>
-      </c>
-      <c r="N46" t="inlineStr"/>
+        <v>2026</v>
+      </c>
+      <c r="N46" t="n">
+        <v>122</v>
+      </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>WATERENVIRONMENT_SFTDN</t>
+          <t>Vannmiljø</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
@@ -3283,7 +3279,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>002-3659-R</t>
+          <t>002-3685-R</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3293,12 +3289,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>QE3-1-6-2 - Phosphorus Conditions</t>
+          <t>QE3-1-6-1 - Nitrogen conditions</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Orthophosphate</t>
+          <t>Total oxidised Nitrogen</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -3309,7 +3305,7 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="n">
-        <v>46.070588</v>
+        <v>592</v>
       </c>
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr">
@@ -3319,14 +3315,12 @@
       </c>
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="n">
-        <v>2020</v>
+        <v>2014</v>
       </c>
       <c r="M47" t="n">
-        <v>2025</v>
-      </c>
-      <c r="N47" t="n">
-        <v>68</v>
-      </c>
+        <v>2017</v>
+      </c>
+      <c r="N47" t="inlineStr"/>
       <c r="O47" t="inlineStr">
         <is>
           <t>Vannmiljø</t>
@@ -3341,7 +3335,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>002-3659-R</t>
+          <t>002-3685-R</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -3356,36 +3350,34 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Total phosphorous</t>
+          <t>Orthophosphate</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Not classified</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
-      <c r="G48" t="n">
-        <v>0.3</v>
-      </c>
+      <c r="G48" t="inlineStr"/>
       <c r="H48" t="n">
-        <v>94.451612</v>
+        <v>33.579761</v>
       </c>
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr">
         <is>
-          <t>µg/l P</t>
+          <t>µg/l</t>
         </is>
       </c>
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="M48" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="N48" t="n">
-        <v>186</v>
+        <v>84</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>
@@ -3401,7 +3393,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>002-3659-R</t>
+          <t>002-3685-R</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -3416,23 +3408,25 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Phosphate</t>
+          <t>Total phosphorous</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Not classified</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
+      <c r="G49" t="n">
+        <v>0.5</v>
+      </c>
       <c r="H49" t="n">
-        <v>67.820212</v>
+        <v>64.364</v>
       </c>
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr">
         <is>
-          <t>µg/l</t>
+          <t>µg/l P</t>
         </is>
       </c>
       <c r="K49" t="inlineStr"/>
@@ -3440,10 +3434,10 @@
         <v>2020</v>
       </c>
       <c r="M49" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="N49" t="n">
-        <v>94</v>
+        <v>125</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
@@ -3459,7 +3453,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>002-599-R</t>
+          <t>002-3685-R</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3469,49 +3463,39 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>QE3-1-6-1 - Nitrogen conditions</t>
+          <t>QE3-1-6-2 - Phosphorus Conditions</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Ammonia</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Poor</t>
-        </is>
-      </c>
-      <c r="F50" t="n">
-        <v>0.06900000000000001</v>
-      </c>
-      <c r="G50" t="n">
-        <v>0.2347</v>
-      </c>
+          <t>Not classified</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
       <c r="H50" t="n">
-        <v>145</v>
-      </c>
-      <c r="I50" t="n">
-        <v>10</v>
-      </c>
+        <v>34.871028</v>
+      </c>
+      <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr">
         <is>
           <t>µg/l</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>30.0;60.0;100.0;160.0</t>
-        </is>
-      </c>
+      <c r="K50" t="inlineStr"/>
       <c r="L50" t="n">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="M50" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="N50" t="n">
-        <v>6</v>
+        <v>107</v>
       </c>
       <c r="O50" t="inlineStr">
         <is>
@@ -3527,7 +3511,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>002-599-R</t>
+          <t>002-3687-R</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3542,25 +3526,25 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Total nitrogen</t>
+          <t>Ammonia</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Bad</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>0.1229</v>
+        <v>0.1524</v>
       </c>
       <c r="G51" t="n">
-        <v>0.1531</v>
+        <v>0.5571</v>
       </c>
       <c r="H51" t="n">
-        <v>2645.257731</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="I51" t="n">
-        <v>325</v>
+        <v>10</v>
       </c>
       <c r="J51" t="inlineStr">
         <is>
@@ -3569,21 +3553,19 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>550.0;775.0;1325.0;2025.0</t>
+          <t>30.0;60.0;100.0;160.0</t>
         </is>
       </c>
       <c r="L51" t="n">
-        <v>2019</v>
+        <v>2014</v>
       </c>
       <c r="M51" t="n">
-        <v>2025</v>
-      </c>
-      <c r="N51" t="n">
-        <v>97</v>
-      </c>
+        <v>2014</v>
+      </c>
+      <c r="N51" t="inlineStr"/>
       <c r="O51" t="inlineStr">
         <is>
-          <t>Vannmiljø</t>
+          <t>VannMiljø</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
@@ -3595,7 +3577,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>002-599-R</t>
+          <t>002-3687-R</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -3610,34 +3592,44 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Total organic carbon</t>
+          <t>Total nitrogen</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Not classified</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>0.3663</v>
+      </c>
+      <c r="G52" t="n">
+        <v>0.539</v>
+      </c>
       <c r="H52" t="n">
-        <v>9.52</v>
-      </c>
-      <c r="I52" t="inlineStr"/>
+        <v>887.260869</v>
+      </c>
+      <c r="I52" t="n">
+        <v>325</v>
+      </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>mg/l C</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr"/>
+          <t>µg/l</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>550.0;775.0;1325.0;2025.0</t>
+        </is>
+      </c>
       <c r="L52" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="M52" t="n">
         <v>2025</v>
       </c>
       <c r="N52" t="n">
-        <v>91</v>
+        <v>46</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
@@ -3653,7 +3645,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>002-599-R</t>
+          <t>002-3687-R</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -3668,7 +3660,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Total oxidised Nitrogen</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -3679,7 +3671,7 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="n">
-        <v>1578.333333</v>
+        <v>29.797297</v>
       </c>
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr">
@@ -3689,13 +3681,13 @@
       </c>
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="n">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="M53" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="N53" t="n">
-        <v>6</v>
+        <v>37</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
@@ -3711,7 +3703,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>002-599-R</t>
+          <t>002-3687-R</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3721,41 +3713,39 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>QE3-1-6-2 - Phosphorus Conditions</t>
+          <t>QE3-1-6-1 - Nitrogen conditions</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Orthophosphate</t>
+          <t>Total organic carbon</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Not classified</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
-      <c r="G54" t="n">
-        <v>0.5</v>
-      </c>
+      <c r="G54" t="inlineStr"/>
       <c r="H54" t="n">
-        <v>60.289473</v>
+        <v>15.272727</v>
       </c>
       <c r="I54" t="inlineStr"/>
       <c r="J54" t="inlineStr">
         <is>
-          <t>µg/l</t>
+          <t>mg/l C</t>
         </is>
       </c>
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="M54" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="N54" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="O54" t="inlineStr">
         <is>
@@ -3771,7 +3761,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>002-599-R</t>
+          <t>002-3687-R</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3781,41 +3771,39 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>QE3-1-6-2 - Phosphorus Conditions</t>
+          <t>QE3-1-6-1 - Nitrogen conditions</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Total phosphorous</t>
+          <t>Total oxidised Nitrogen</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Not classified</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
-      <c r="G55" t="n">
-        <v>0.5</v>
-      </c>
+      <c r="G55" t="inlineStr"/>
       <c r="H55" t="n">
-        <v>83.15000000000001</v>
+        <v>480</v>
       </c>
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr">
         <is>
-          <t>µg/l P</t>
+          <t>µg/l</t>
         </is>
       </c>
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="n">
-        <v>2019</v>
+        <v>2017</v>
       </c>
       <c r="M55" t="n">
-        <v>2025</v>
+        <v>2017</v>
       </c>
       <c r="N55" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="O55" t="inlineStr">
         <is>
@@ -3831,7 +3819,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>002-599-R</t>
+          <t>002-3687-R</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3846,7 +3834,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Phosphate</t>
+          <t>Orthophosphate</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -3857,7 +3845,7 @@
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="n">
-        <v>65.61764700000001</v>
+        <v>28.82</v>
       </c>
       <c r="I56" t="inlineStr"/>
       <c r="J56" t="inlineStr">
@@ -3867,13 +3855,13 @@
       </c>
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="M56" t="n">
         <v>2025</v>
       </c>
       <c r="N56" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
@@ -3889,7 +3877,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>002-3685-R</t>
+          <t>002-3687-R</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3899,12 +3887,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>QE3-1-6-1 - Nitrogen conditions</t>
+          <t>QE3-1-6-2 - Phosphorus Conditions</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Ammonia</t>
+          <t>Total phosphorous</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -3912,38 +3900,32 @@
           <t>Moderate</t>
         </is>
       </c>
-      <c r="F57" t="n">
-        <v>0.1524</v>
-      </c>
+      <c r="F57" t="inlineStr"/>
       <c r="G57" t="n">
-        <v>0.5571</v>
+        <v>0.5</v>
       </c>
       <c r="H57" t="n">
-        <v>65.59999999999999</v>
-      </c>
-      <c r="I57" t="n">
-        <v>10</v>
-      </c>
+        <v>60.234042</v>
+      </c>
+      <c r="I57" t="inlineStr"/>
       <c r="J57" t="inlineStr">
         <is>
-          <t>µg/l</t>
-        </is>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>30.0;60.0;100.0;160.0</t>
-        </is>
-      </c>
+          <t>µg/l P</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr"/>
       <c r="L57" t="n">
-        <v>2014</v>
+        <v>2020</v>
       </c>
       <c r="M57" t="n">
-        <v>2014</v>
-      </c>
-      <c r="N57" t="inlineStr"/>
+        <v>2025</v>
+      </c>
+      <c r="N57" t="n">
+        <v>47</v>
+      </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>VannMiljø</t>
+          <t>Vannmiljø</t>
         </is>
       </c>
       <c r="P57" t="inlineStr">
@@ -3955,7 +3937,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>002-3685-R</t>
+          <t>002-3687-R</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3965,49 +3947,39 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>QE3-1-6-1 - Nitrogen conditions</t>
+          <t>QE3-1-6-2 - Phosphorus Conditions</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Total nitrogen</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="F58" t="n">
-        <v>0.2474</v>
-      </c>
-      <c r="G58" t="n">
-        <v>0.4024</v>
-      </c>
+          <t>Not classified</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
       <c r="H58" t="n">
-        <v>1313.451612</v>
-      </c>
-      <c r="I58" t="n">
-        <v>325</v>
-      </c>
+        <v>29.797297</v>
+      </c>
+      <c r="I58" t="inlineStr"/>
       <c r="J58" t="inlineStr">
         <is>
           <t>µg/l</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>550.0;775.0;1325.0;2025.0</t>
-        </is>
-      </c>
+      <c r="K58" t="inlineStr"/>
       <c r="L58" t="n">
         <v>2020</v>
       </c>
       <c r="M58" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="N58" t="n">
-        <v>124</v>
+        <v>37</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
@@ -4023,7 +3995,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>002-3685-R</t>
+          <t>002-3655-R</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -4038,34 +4010,44 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Phosphate</t>
+          <t>Total nitrogen</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Not classified</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>0.377</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0.5513</v>
+      </c>
       <c r="H59" t="n">
-        <v>34.871028</v>
-      </c>
-      <c r="I59" t="inlineStr"/>
+        <v>861.961038</v>
+      </c>
+      <c r="I59" t="n">
+        <v>325</v>
+      </c>
       <c r="J59" t="inlineStr">
         <is>
           <t>µg/l</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr"/>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>550.0;775.0;1325.0;2025.0</t>
+        </is>
+      </c>
       <c r="L59" t="n">
         <v>2020</v>
       </c>
       <c r="M59" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="N59" t="n">
-        <v>107</v>
+        <v>154</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
@@ -4081,7 +4063,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>002-3685-R</t>
+          <t>002-3655-R</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -4096,7 +4078,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Total organic carbon</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -4107,12 +4089,12 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="n">
-        <v>13.990163</v>
+        <v>17.5288</v>
       </c>
       <c r="I60" t="inlineStr"/>
       <c r="J60" t="inlineStr">
         <is>
-          <t>mg/l C</t>
+          <t>µg/l</t>
         </is>
       </c>
       <c r="K60" t="inlineStr"/>
@@ -4120,10 +4102,10 @@
         <v>2020</v>
       </c>
       <c r="M60" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="N60" t="n">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
@@ -4139,7 +4121,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>002-3685-R</t>
+          <t>002-3655-R</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -4154,7 +4136,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Total oxidised Nitrogen</t>
+          <t>Total organic carbon</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -4165,22 +4147,24 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="n">
-        <v>592</v>
+        <v>12.721333</v>
       </c>
       <c r="I61" t="inlineStr"/>
       <c r="J61" t="inlineStr">
         <is>
-          <t>µg/l</t>
+          <t>mg/l C</t>
         </is>
       </c>
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="n">
-        <v>2014</v>
+        <v>2020</v>
       </c>
       <c r="M61" t="n">
-        <v>2017</v>
-      </c>
-      <c r="N61" t="inlineStr"/>
+        <v>2026</v>
+      </c>
+      <c r="N61" t="n">
+        <v>150</v>
+      </c>
       <c r="O61" t="inlineStr">
         <is>
           <t>Vannmiljø</t>
@@ -4195,7 +4179,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>002-3685-R</t>
+          <t>002-3655-R</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -4205,12 +4189,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>QE3-1-6-2 - Phosphorus Conditions</t>
+          <t>QE3-1-6-1 - Nitrogen conditions</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Orthophosphate</t>
+          <t>Total oxidised Nitrogen</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -4221,7 +4205,7 @@
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="n">
-        <v>33.579761</v>
+        <v>30</v>
       </c>
       <c r="I62" t="inlineStr"/>
       <c r="J62" t="inlineStr">
@@ -4231,13 +4215,13 @@
       </c>
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="n">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="M62" t="n">
-        <v>2025</v>
+        <v>2019</v>
       </c>
       <c r="N62" t="n">
-        <v>84</v>
+        <v>2</v>
       </c>
       <c r="O62" t="inlineStr">
         <is>
@@ -4253,7 +4237,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>002-3685-R</t>
+          <t>002-3655-R</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -4268,36 +4252,34 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Total phosphorous</t>
+          <t>Orthophosphate</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Not classified</t>
         </is>
       </c>
       <c r="F63" t="inlineStr"/>
-      <c r="G63" t="n">
-        <v>0.5</v>
-      </c>
+      <c r="G63" t="inlineStr"/>
       <c r="H63" t="n">
-        <v>64.364</v>
+        <v>15.63238</v>
       </c>
       <c r="I63" t="inlineStr"/>
       <c r="J63" t="inlineStr">
         <is>
-          <t>µg/l P</t>
+          <t>µg/l</t>
         </is>
       </c>
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="M63" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="N63" t="n">
-        <v>125</v>
+        <v>105</v>
       </c>
       <c r="O63" t="inlineStr">
         <is>
@@ -4313,7 +4295,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>002-3685-R</t>
+          <t>002-3655-R</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -4328,34 +4310,44 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Phosphate</t>
+          <t>Total phosphorous</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Not classified</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>0.3241</v>
+      </c>
+      <c r="G64" t="n">
+        <v>0.5417999999999999</v>
+      </c>
       <c r="H64" t="n">
-        <v>34.871028</v>
-      </c>
-      <c r="I64" t="inlineStr"/>
+        <v>33.944516</v>
+      </c>
+      <c r="I64" t="n">
+        <v>11</v>
+      </c>
       <c r="J64" t="inlineStr">
         <is>
           <t>µg/l</t>
         </is>
       </c>
-      <c r="K64" t="inlineStr"/>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>20.0;29.0;58.0;98.0</t>
+        </is>
+      </c>
       <c r="L64" t="n">
         <v>2020</v>
       </c>
       <c r="M64" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="N64" t="n">
-        <v>107</v>
+        <v>155</v>
       </c>
       <c r="O64" t="inlineStr">
         <is>
@@ -4371,7 +4363,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>002-3687-R</t>
+          <t>002-3655-R</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -4381,898 +4373,46 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>QE3-1-6-1 - Nitrogen conditions</t>
+          <t>QE3-1-6-2 - Phosphorus Conditions</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Ammonia</t>
+          <t>Phosphate</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="F65" t="n">
-        <v>0.1524</v>
-      </c>
-      <c r="G65" t="n">
-        <v>0.5571</v>
-      </c>
+          <t>Not classified</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
       <c r="H65" t="n">
-        <v>65.59999999999999</v>
-      </c>
-      <c r="I65" t="n">
-        <v>10</v>
-      </c>
+        <v>17.5288</v>
+      </c>
+      <c r="I65" t="inlineStr"/>
       <c r="J65" t="inlineStr">
         <is>
           <t>µg/l</t>
         </is>
       </c>
-      <c r="K65" t="inlineStr">
-        <is>
-          <t>30.0;60.0;100.0;160.0</t>
-        </is>
-      </c>
+      <c r="K65" t="inlineStr"/>
       <c r="L65" t="n">
-        <v>2014</v>
+        <v>2020</v>
       </c>
       <c r="M65" t="n">
-        <v>2014</v>
-      </c>
-      <c r="N65" t="inlineStr"/>
+        <v>2025</v>
+      </c>
+      <c r="N65" t="n">
+        <v>125</v>
+      </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>VannMiljø</t>
+          <t>Vannmiljø</t>
         </is>
       </c>
       <c r="P65" t="inlineStr">
-        <is>
-          <t>Measured</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>002-3687-R</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>PhysicoChemical</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>QE3-1-6-1 - Nitrogen conditions</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>Total nitrogen</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="F66" t="n">
-        <v>0.3663</v>
-      </c>
-      <c r="G66" t="n">
-        <v>0.539</v>
-      </c>
-      <c r="H66" t="n">
-        <v>887.260869</v>
-      </c>
-      <c r="I66" t="n">
-        <v>325</v>
-      </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>µg/l</t>
-        </is>
-      </c>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t>550.0;775.0;1325.0;2025.0</t>
-        </is>
-      </c>
-      <c r="L66" t="n">
-        <v>2020</v>
-      </c>
-      <c r="M66" t="n">
-        <v>2025</v>
-      </c>
-      <c r="N66" t="n">
-        <v>46</v>
-      </c>
-      <c r="O66" t="inlineStr">
-        <is>
-          <t>Vannmiljø</t>
-        </is>
-      </c>
-      <c r="P66" t="inlineStr">
-        <is>
-          <t>Measured</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>002-3687-R</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>PhysicoChemical</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>QE3-1-6-1 - Nitrogen conditions</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>Phosphate</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>Not classified</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="n">
-        <v>29.797297</v>
-      </c>
-      <c r="I67" t="inlineStr"/>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>µg/l</t>
-        </is>
-      </c>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="n">
-        <v>2020</v>
-      </c>
-      <c r="M67" t="n">
-        <v>2025</v>
-      </c>
-      <c r="N67" t="n">
-        <v>37</v>
-      </c>
-      <c r="O67" t="inlineStr">
-        <is>
-          <t>Vannmiljø</t>
-        </is>
-      </c>
-      <c r="P67" t="inlineStr">
-        <is>
-          <t>Measured</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>002-3687-R</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>PhysicoChemical</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>QE3-1-6-1 - Nitrogen conditions</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>Total organic carbon</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>Not classified</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr"/>
-      <c r="H68" t="n">
-        <v>15.272727</v>
-      </c>
-      <c r="I68" t="inlineStr"/>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>mg/l C</t>
-        </is>
-      </c>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="n">
-        <v>2020</v>
-      </c>
-      <c r="M68" t="n">
-        <v>2025</v>
-      </c>
-      <c r="N68" t="n">
-        <v>44</v>
-      </c>
-      <c r="O68" t="inlineStr">
-        <is>
-          <t>Vannmiljø</t>
-        </is>
-      </c>
-      <c r="P68" t="inlineStr">
-        <is>
-          <t>Measured</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>002-3687-R</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>PhysicoChemical</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>QE3-1-6-1 - Nitrogen conditions</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>Total oxidised Nitrogen</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>Not classified</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr"/>
-      <c r="H69" t="n">
-        <v>480</v>
-      </c>
-      <c r="I69" t="inlineStr"/>
-      <c r="J69" t="inlineStr">
-        <is>
-          <t>µg/l</t>
-        </is>
-      </c>
-      <c r="K69" t="inlineStr"/>
-      <c r="L69" t="n">
-        <v>2017</v>
-      </c>
-      <c r="M69" t="n">
-        <v>2017</v>
-      </c>
-      <c r="N69" t="n">
-        <v>1</v>
-      </c>
-      <c r="O69" t="inlineStr">
-        <is>
-          <t>Vannmiljø</t>
-        </is>
-      </c>
-      <c r="P69" t="inlineStr">
-        <is>
-          <t>Measured</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>002-3687-R</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>PhysicoChemical</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>QE3-1-6-2 - Phosphorus Conditions</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>Orthophosphate</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>Not classified</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr"/>
-      <c r="H70" t="n">
-        <v>28.82</v>
-      </c>
-      <c r="I70" t="inlineStr"/>
-      <c r="J70" t="inlineStr">
-        <is>
-          <t>µg/l</t>
-        </is>
-      </c>
-      <c r="K70" t="inlineStr"/>
-      <c r="L70" t="n">
-        <v>2021</v>
-      </c>
-      <c r="M70" t="n">
-        <v>2025</v>
-      </c>
-      <c r="N70" t="n">
-        <v>30</v>
-      </c>
-      <c r="O70" t="inlineStr">
-        <is>
-          <t>Vannmiljø</t>
-        </is>
-      </c>
-      <c r="P70" t="inlineStr">
-        <is>
-          <t>Measured</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>002-3687-R</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>PhysicoChemical</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>QE3-1-6-2 - Phosphorus Conditions</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>Total phosphorous</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr"/>
-      <c r="G71" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="H71" t="n">
-        <v>60.234042</v>
-      </c>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>µg/l P</t>
-        </is>
-      </c>
-      <c r="K71" t="inlineStr"/>
-      <c r="L71" t="n">
-        <v>2020</v>
-      </c>
-      <c r="M71" t="n">
-        <v>2025</v>
-      </c>
-      <c r="N71" t="n">
-        <v>47</v>
-      </c>
-      <c r="O71" t="inlineStr">
-        <is>
-          <t>Vannmiljø</t>
-        </is>
-      </c>
-      <c r="P71" t="inlineStr">
-        <is>
-          <t>Measured</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>002-3687-R</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>PhysicoChemical</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>QE3-1-6-2 - Phosphorus Conditions</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>Phosphate</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>Not classified</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr"/>
-      <c r="H72" t="n">
-        <v>29.797297</v>
-      </c>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr">
-        <is>
-          <t>µg/l</t>
-        </is>
-      </c>
-      <c r="K72" t="inlineStr"/>
-      <c r="L72" t="n">
-        <v>2020</v>
-      </c>
-      <c r="M72" t="n">
-        <v>2025</v>
-      </c>
-      <c r="N72" t="n">
-        <v>37</v>
-      </c>
-      <c r="O72" t="inlineStr">
-        <is>
-          <t>Vannmiljø</t>
-        </is>
-      </c>
-      <c r="P72" t="inlineStr">
-        <is>
-          <t>Measured</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>002-3655-R</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>PhysicoChemical</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>QE3-1-6-1 - Nitrogen conditions</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>Total nitrogen</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="F73" t="n">
-        <v>0.377</v>
-      </c>
-      <c r="G73" t="n">
-        <v>0.5513</v>
-      </c>
-      <c r="H73" t="n">
-        <v>861.961038</v>
-      </c>
-      <c r="I73" t="n">
-        <v>325</v>
-      </c>
-      <c r="J73" t="inlineStr">
-        <is>
-          <t>µg/l</t>
-        </is>
-      </c>
-      <c r="K73" t="inlineStr">
-        <is>
-          <t>550.0;775.0;1325.0;2025.0</t>
-        </is>
-      </c>
-      <c r="L73" t="n">
-        <v>2020</v>
-      </c>
-      <c r="M73" t="n">
-        <v>2026</v>
-      </c>
-      <c r="N73" t="n">
-        <v>154</v>
-      </c>
-      <c r="O73" t="inlineStr">
-        <is>
-          <t>Vannmiljø</t>
-        </is>
-      </c>
-      <c r="P73" t="inlineStr">
-        <is>
-          <t>Measured</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>002-3655-R</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>PhysicoChemical</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>QE3-1-6-1 - Nitrogen conditions</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>Phosphate</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>Not classified</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr"/>
-      <c r="H74" t="n">
-        <v>17.5288</v>
-      </c>
-      <c r="I74" t="inlineStr"/>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>µg/l</t>
-        </is>
-      </c>
-      <c r="K74" t="inlineStr"/>
-      <c r="L74" t="n">
-        <v>2020</v>
-      </c>
-      <c r="M74" t="n">
-        <v>2025</v>
-      </c>
-      <c r="N74" t="n">
-        <v>125</v>
-      </c>
-      <c r="O74" t="inlineStr">
-        <is>
-          <t>Vannmiljø</t>
-        </is>
-      </c>
-      <c r="P74" t="inlineStr">
-        <is>
-          <t>Measured</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>002-3655-R</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>PhysicoChemical</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>QE3-1-6-1 - Nitrogen conditions</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>Total organic carbon</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>Not classified</t>
-        </is>
-      </c>
-      <c r="F75" t="inlineStr"/>
-      <c r="G75" t="inlineStr"/>
-      <c r="H75" t="n">
-        <v>12.721333</v>
-      </c>
-      <c r="I75" t="inlineStr"/>
-      <c r="J75" t="inlineStr">
-        <is>
-          <t>mg/l C</t>
-        </is>
-      </c>
-      <c r="K75" t="inlineStr"/>
-      <c r="L75" t="n">
-        <v>2020</v>
-      </c>
-      <c r="M75" t="n">
-        <v>2026</v>
-      </c>
-      <c r="N75" t="n">
-        <v>150</v>
-      </c>
-      <c r="O75" t="inlineStr">
-        <is>
-          <t>Vannmiljø</t>
-        </is>
-      </c>
-      <c r="P75" t="inlineStr">
-        <is>
-          <t>Measured</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>002-3655-R</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>PhysicoChemical</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>QE3-1-6-1 - Nitrogen conditions</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>Total oxidised Nitrogen</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>Not classified</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr"/>
-      <c r="G76" t="inlineStr"/>
-      <c r="H76" t="n">
-        <v>30</v>
-      </c>
-      <c r="I76" t="inlineStr"/>
-      <c r="J76" t="inlineStr">
-        <is>
-          <t>µg/l</t>
-        </is>
-      </c>
-      <c r="K76" t="inlineStr"/>
-      <c r="L76" t="n">
-        <v>2019</v>
-      </c>
-      <c r="M76" t="n">
-        <v>2019</v>
-      </c>
-      <c r="N76" t="n">
-        <v>2</v>
-      </c>
-      <c r="O76" t="inlineStr">
-        <is>
-          <t>Vannmiljø</t>
-        </is>
-      </c>
-      <c r="P76" t="inlineStr">
-        <is>
-          <t>Measured</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>002-3655-R</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>PhysicoChemical</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>QE3-1-6-2 - Phosphorus Conditions</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>Orthophosphate</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>Not classified</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr"/>
-      <c r="G77" t="inlineStr"/>
-      <c r="H77" t="n">
-        <v>15.63238</v>
-      </c>
-      <c r="I77" t="inlineStr"/>
-      <c r="J77" t="inlineStr">
-        <is>
-          <t>µg/l</t>
-        </is>
-      </c>
-      <c r="K77" t="inlineStr"/>
-      <c r="L77" t="n">
-        <v>2021</v>
-      </c>
-      <c r="M77" t="n">
-        <v>2025</v>
-      </c>
-      <c r="N77" t="n">
-        <v>105</v>
-      </c>
-      <c r="O77" t="inlineStr">
-        <is>
-          <t>Vannmiljø</t>
-        </is>
-      </c>
-      <c r="P77" t="inlineStr">
-        <is>
-          <t>Measured</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>002-3655-R</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>PhysicoChemical</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>QE3-1-6-2 - Phosphorus Conditions</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>Total phosphorous</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
-      <c r="F78" t="n">
-        <v>0.3241</v>
-      </c>
-      <c r="G78" t="n">
-        <v>0.5417999999999999</v>
-      </c>
-      <c r="H78" t="n">
-        <v>33.944516</v>
-      </c>
-      <c r="I78" t="n">
-        <v>11</v>
-      </c>
-      <c r="J78" t="inlineStr">
-        <is>
-          <t>µg/l</t>
-        </is>
-      </c>
-      <c r="K78" t="inlineStr">
-        <is>
-          <t>20.0;29.0;58.0;98.0</t>
-        </is>
-      </c>
-      <c r="L78" t="n">
-        <v>2020</v>
-      </c>
-      <c r="M78" t="n">
-        <v>2026</v>
-      </c>
-      <c r="N78" t="n">
-        <v>155</v>
-      </c>
-      <c r="O78" t="inlineStr">
-        <is>
-          <t>Vannmiljø</t>
-        </is>
-      </c>
-      <c r="P78" t="inlineStr">
-        <is>
-          <t>Measured</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>002-3655-R</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>PhysicoChemical</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>QE3-1-6-2 - Phosphorus Conditions</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>Phosphate</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>Not classified</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr"/>
-      <c r="G79" t="inlineStr"/>
-      <c r="H79" t="n">
-        <v>17.5288</v>
-      </c>
-      <c r="I79" t="inlineStr"/>
-      <c r="J79" t="inlineStr">
-        <is>
-          <t>µg/l</t>
-        </is>
-      </c>
-      <c r="K79" t="inlineStr"/>
-      <c r="L79" t="n">
-        <v>2020</v>
-      </c>
-      <c r="M79" t="n">
-        <v>2025</v>
-      </c>
-      <c r="N79" t="n">
-        <v>125</v>
-      </c>
-      <c r="O79" t="inlineStr">
-        <is>
-          <t>Vannmiljø</t>
-        </is>
-      </c>
-      <c r="P79" t="inlineStr">
         <is>
           <t>Measured</t>
         </is>

</xml_diff>